<commit_message>
Refactoring majeur : architecture OOP + énumération améliorée
- Introduit RelaySolution, RelayModel, RelayConstraints, RelaySolver
  comme API centrales (remplace constraint_model / solution_formatter)
- Refactorise enumerate.py avec RelayModel et RelaySolution ;
  renomme le dossier de sortie en enumerate_solutions/
- Ajoute export JSON des solutions et calcul de rest_h dans solver
- Remplace l'objectif (count binômes → somme pondérée des scores)
- Réécrit verifications.py : check() prend list[dict] + RelayConstraints
- Implémente RelaySolver en itérateur streaming (thread + queue)
- Extrait RelayConstraints dans constraints.py
- Améliore le rendu HTML (tables natives, stats, formatage .1f)
- Supprime upper_bound.py et le code dupliqué dans analyze_solutions
- Active les contraintes de dispos et binômes ;
- Active ENABLE_FLEXIBILITY ; compatibilité coureurs multi-niveaux
- Met à jour CLAUDE.md et README.md
</commit_message>
<xml_diff>
--- a/compat_coureurs.xlsx
+++ b/compat_coureurs.xlsx
@@ -5,18 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j46951\Documents\relay-planner\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://edfonline-my.sharepoint.com/personal/vincent_champouillon_edf_fr/Documents/Python/relay-planner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{DAC89DCA-730F-49DF-8B02-04F14E485EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="101" documentId="8_{404F38C6-A597-48AD-A233-0E34BD6AF467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22D95CA8-01B4-41D2-9D16-67FB895DDA3C}"/>
   <bookViews>
-    <workbookView xWindow="-27240" yWindow="810" windowWidth="26400" windowHeight="13110" xr2:uid="{A099FB4B-584E-424D-AA06-C43916DCFDF2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A099FB4B-584E-424D-AA06-C43916DCFDF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="15">
   <si>
     <t>Pierre</t>
   </si>
@@ -82,12 +81,6 @@
   </si>
   <si>
     <t>X</t>
-  </si>
-  <si>
-    <t>Oui</t>
-  </si>
-  <si>
-    <t>Non</t>
   </si>
 </sst>
 </file>
@@ -595,9 +588,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0F2359D-AA5F-4280-907D-24A78CC77484}">
   <dimension ref="B4:P18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B4" s="5"/>
       <c r="C4" s="8" t="s">
         <v>0</v>
@@ -642,7 +635,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B5" s="6" t="s">
         <v>0</v>
       </c>
@@ -663,12 +656,12 @@
       <c r="O5" s="1"/>
       <c r="P5" s="2"/>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>15</v>
+      <c r="C6" s="1">
+        <v>2</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>14</v>
@@ -686,15 +679,15 @@
       <c r="O6" s="1"/>
       <c r="P6" s="2"/>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>15</v>
+      <c r="C7" s="1">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1">
+        <v>2</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>14</v>
@@ -711,18 +704,18 @@
       <c r="O7" s="1"/>
       <c r="P7" s="2"/>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>15</v>
+      <c r="C8" s="1">
+        <v>2</v>
+      </c>
+      <c r="D8" s="1">
+        <v>2</v>
+      </c>
+      <c r="E8" s="1">
+        <v>2</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>14</v>
@@ -738,21 +731,21 @@
       <c r="O8" s="1"/>
       <c r="P8" s="2"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B9" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>15</v>
+      <c r="C9" s="1">
+        <v>2</v>
+      </c>
+      <c r="D9" s="1">
+        <v>2</v>
+      </c>
+      <c r="E9" s="1">
+        <v>2</v>
+      </c>
+      <c r="F9" s="1">
+        <v>2</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>14</v>
@@ -767,24 +760,24 @@
       <c r="O9" s="1"/>
       <c r="P9" s="2"/>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B10" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>15</v>
+      <c r="C10" s="1">
+        <v>2</v>
+      </c>
+      <c r="D10" s="1">
+        <v>2</v>
+      </c>
+      <c r="E10" s="1">
+        <v>2</v>
+      </c>
+      <c r="F10" s="1">
+        <v>2</v>
+      </c>
+      <c r="G10" s="1">
+        <v>2</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>14</v>
@@ -798,27 +791,27 @@
       <c r="O10" s="1"/>
       <c r="P10" s="2"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B11" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>15</v>
+      <c r="C11" s="1">
+        <v>2</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2</v>
+      </c>
+      <c r="E11" s="1">
+        <v>2</v>
+      </c>
+      <c r="F11" s="1">
+        <v>2</v>
+      </c>
+      <c r="G11" s="1">
+        <v>2</v>
+      </c>
+      <c r="H11" s="1">
+        <v>1</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>14</v>
@@ -831,30 +824,30 @@
       <c r="O11" s="1"/>
       <c r="P11" s="2"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>15</v>
+      <c r="C12" s="1">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1">
+        <v>2</v>
+      </c>
+      <c r="E12" s="1">
+        <v>2</v>
+      </c>
+      <c r="F12" s="1">
+        <v>2</v>
+      </c>
+      <c r="G12" s="1">
+        <v>2</v>
+      </c>
+      <c r="H12" s="1">
+        <v>1</v>
+      </c>
+      <c r="I12" s="1">
+        <v>2</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>14</v>
@@ -866,33 +859,33 @@
       <c r="O12" s="1"/>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B13" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>15</v>
+      <c r="C13" s="1">
+        <v>2</v>
+      </c>
+      <c r="D13" s="1">
+        <v>2</v>
+      </c>
+      <c r="E13" s="1">
+        <v>2</v>
+      </c>
+      <c r="F13" s="1">
+        <v>2</v>
+      </c>
+      <c r="G13" s="1">
+        <v>2</v>
+      </c>
+      <c r="H13" s="1">
+        <v>1</v>
+      </c>
+      <c r="I13" s="1">
+        <v>2</v>
+      </c>
+      <c r="J13" s="1">
+        <v>2</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>14</v>
@@ -903,36 +896,36 @@
       <c r="O13" s="1"/>
       <c r="P13" s="2"/>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>15</v>
+      <c r="C14" s="1">
+        <v>2</v>
+      </c>
+      <c r="D14" s="1">
+        <v>2</v>
+      </c>
+      <c r="E14" s="1">
+        <v>2</v>
+      </c>
+      <c r="F14" s="1">
+        <v>2</v>
+      </c>
+      <c r="G14" s="1">
+        <v>2</v>
+      </c>
+      <c r="H14" s="1">
+        <v>1</v>
+      </c>
+      <c r="I14" s="1">
+        <v>2</v>
+      </c>
+      <c r="J14" s="1">
+        <v>2</v>
+      </c>
+      <c r="K14" s="1">
+        <v>2</v>
       </c>
       <c r="L14" s="1" t="s">
         <v>14</v>
@@ -942,39 +935,39 @@
       <c r="O14" s="1"/>
       <c r="P14" s="2"/>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B15" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>15</v>
+      <c r="C15" s="1">
+        <v>2</v>
+      </c>
+      <c r="D15" s="1">
+        <v>2</v>
+      </c>
+      <c r="E15" s="1">
+        <v>2</v>
+      </c>
+      <c r="F15" s="1">
+        <v>2</v>
+      </c>
+      <c r="G15" s="1">
+        <v>2</v>
+      </c>
+      <c r="H15" s="1">
+        <v>1</v>
+      </c>
+      <c r="I15" s="1">
+        <v>2</v>
+      </c>
+      <c r="J15" s="1">
+        <v>2</v>
+      </c>
+      <c r="K15" s="1">
+        <v>2</v>
+      </c>
+      <c r="L15" s="1">
+        <v>2</v>
       </c>
       <c r="M15" s="1" t="s">
         <v>14</v>
@@ -983,42 +976,42 @@
       <c r="O15" s="1"/>
       <c r="P15" s="2"/>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>16</v>
+      <c r="C16" s="1">
+        <v>1</v>
+      </c>
+      <c r="D16" s="1">
+        <v>2</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+      <c r="F16" s="1">
+        <v>2</v>
+      </c>
+      <c r="G16" s="1">
+        <v>2</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>1</v>
+      </c>
+      <c r="J16" s="1">
+        <v>2</v>
+      </c>
+      <c r="K16" s="1">
+        <v>2</v>
+      </c>
+      <c r="L16" s="1">
+        <v>2</v>
+      </c>
+      <c r="M16" s="1">
+        <v>1</v>
       </c>
       <c r="N16" s="1" t="s">
         <v>14</v>
@@ -1026,93 +1019,93 @@
       <c r="O16" s="1"/>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L17" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="N17" s="1" t="s">
-        <v>15</v>
+      <c r="C17" s="1">
+        <v>0</v>
+      </c>
+      <c r="D17" s="1">
+        <v>2</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1">
+        <v>1</v>
+      </c>
+      <c r="G17" s="1">
+        <v>1</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1</v>
+      </c>
+      <c r="J17" s="1">
+        <v>2</v>
+      </c>
+      <c r="K17" s="1">
+        <v>1</v>
+      </c>
+      <c r="L17" s="1">
+        <v>1</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="N17" s="1">
+        <v>2</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>14</v>
       </c>
       <c r="P17" s="2"/>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B18" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="N18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="O18" s="3" t="s">
-        <v>15</v>
+      <c r="C18" s="3">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3">
+        <v>1</v>
+      </c>
+      <c r="G18" s="3">
+        <v>1</v>
+      </c>
+      <c r="H18" s="3">
+        <v>0</v>
+      </c>
+      <c r="I18" s="3">
+        <v>1</v>
+      </c>
+      <c r="J18" s="3">
+        <v>1</v>
+      </c>
+      <c r="K18" s="3">
+        <v>0</v>
+      </c>
+      <c r="L18" s="3">
+        <v>0</v>
+      </c>
+      <c r="M18" s="3">
+        <v>0</v>
+      </c>
+      <c r="N18" s="3">
+        <v>0</v>
+      </c>
+      <c r="O18" s="3">
+        <v>2</v>
       </c>
       <c r="P18" s="4" t="s">
         <v>14</v>
@@ -1133,6 +1126,6 @@
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{2d26f538-337a-4593-a7e6-123667b1a538}" enabled="1" method="Standard" siteId="{e242425b-70fc-44dc-9ddf-c21e304e6c80}" contentBits="0" removed="0"/>
+  <clbl:label id="{2d26f538-337a-4593-a7e6-123667b1a538}" enabled="1" method="Standard" siteId="{e242425b-70fc-44dc-9ddf-c21e304e6c80}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Ajout coureur Leo, refactor flexibilité via tuples (req, flex) et nouvel objectif configurable
- Nouveau coureur Leo dans RUNNERS_DATA et matrice de compatibilité mise à jour
- La flexibilité est maintenant encodée par relais via des tuples (nb_seg_requested, nb_seg_flex)
  au lieu d'un booléen flexible par coureur ; le domaine CP-SAT est l'intervalle [min, max]
- Suppression du champ Coureur.flexible ; ENABLE_FLEX reste un flag global
- SOLO_MAX_SIZE et OPTIMISE_SUR ajoutés dans data.py (choix de l'objectif : compat_score,
  distance_solo, flex_minimal)
- model.py : _size_domain et _add_same_relay réécrits pour utiliser les nouveaux tuples ;
  détection de binômes basée sur le chevauchement des domaines de taille
- constraints.py : mise à jour pour propager les nouveaux champs
- refresh_compat.py : robustesse encodage UTF-8 et gestion de Leo
- requirements.txt : ajout dépendance manquante
</commit_message>
<xml_diff>
--- a/compat_coureurs.xlsx
+++ b/compat_coureurs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://edfonline-my.sharepoint.com/personal/vincent_champouillon_edf_fr/Documents/Python/relay-planner/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j46951\Documents\relay-planner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="8_{404F38C6-A597-48AD-A233-0E34BD6AF467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22D95CA8-01B4-41D2-9D16-67FB895DDA3C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADFFC25-398B-4371-A0CB-DD0E0749EB4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A099FB4B-584E-424D-AA06-C43916DCFDF2}"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{A099FB4B-584E-424D-AA06-C43916DCFDF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="16">
   <si>
     <t>Pierre</t>
   </si>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>Leo</t>
   </si>
 </sst>
 </file>
@@ -210,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -231,6 +234,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -587,10 +596,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0F2359D-AA5F-4280-907D-24A78CC77484}">
-  <dimension ref="B4:P18"/>
+  <dimension ref="B4:Q19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B4" s="5"/>
       <c r="C4" s="8" t="s">
         <v>0</v>
@@ -634,8 +643,11 @@
       <c r="P4" s="9" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="Q4" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B5" s="6" t="s">
         <v>0</v>
       </c>
@@ -656,7 +668,7 @@
       <c r="O5" s="1"/>
       <c r="P5" s="2"/>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>1</v>
       </c>
@@ -679,7 +691,7 @@
       <c r="O6" s="1"/>
       <c r="P6" s="2"/>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -704,7 +716,7 @@
       <c r="O7" s="1"/>
       <c r="P7" s="2"/>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
@@ -724,14 +736,18 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
+      <c r="K8" s="1">
+        <v>1</v>
+      </c>
+      <c r="L8" s="1">
+        <v>0</v>
+      </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="2"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B9" s="6" t="s">
         <v>4</v>
       </c>
@@ -760,7 +776,7 @@
       <c r="O9" s="1"/>
       <c r="P9" s="2"/>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B10" s="6" t="s">
         <v>5</v>
       </c>
@@ -791,7 +807,7 @@
       <c r="O10" s="1"/>
       <c r="P10" s="2"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B11" s="6" t="s">
         <v>6</v>
       </c>
@@ -824,7 +840,7 @@
       <c r="O11" s="1"/>
       <c r="P11" s="2"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
@@ -859,7 +875,7 @@
       <c r="O12" s="1"/>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B13" s="6" t="s">
         <v>8</v>
       </c>
@@ -896,7 +912,7 @@
       <c r="O13" s="1"/>
       <c r="P13" s="2"/>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>9</v>
       </c>
@@ -935,7 +951,7 @@
       <c r="O14" s="1"/>
       <c r="P14" s="2"/>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B15" s="6" t="s">
         <v>10</v>
       </c>
@@ -976,7 +992,7 @@
       <c r="O15" s="1"/>
       <c r="P15" s="2"/>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B16" s="6" t="s">
         <v>12</v>
       </c>
@@ -1019,7 +1035,7 @@
       <c r="O16" s="1"/>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B17" s="6" t="s">
         <v>11</v>
       </c>
@@ -1064,7 +1080,7 @@
       </c>
       <c r="P17" s="2"/>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B18" s="7" t="s">
         <v>13</v>
       </c>
@@ -1111,8 +1127,58 @@
         <v>14</v>
       </c>
     </row>
+    <row r="19" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="B19" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="11">
+        <v>0</v>
+      </c>
+      <c r="D19" s="11">
+        <v>2</v>
+      </c>
+      <c r="E19" s="11">
+        <v>1</v>
+      </c>
+      <c r="F19" s="11">
+        <v>1</v>
+      </c>
+      <c r="G19" s="11">
+        <v>1</v>
+      </c>
+      <c r="H19" s="11">
+        <v>0</v>
+      </c>
+      <c r="I19" s="11">
+        <v>1</v>
+      </c>
+      <c r="J19" s="11">
+        <v>1</v>
+      </c>
+      <c r="K19" s="11">
+        <v>1</v>
+      </c>
+      <c r="L19" s="11">
+        <v>1</v>
+      </c>
+      <c r="M19" s="11">
+        <v>0</v>
+      </c>
+      <c r="N19" s="11">
+        <v>2</v>
+      </c>
+      <c r="O19" s="11">
+        <v>2</v>
+      </c>
+      <c r="P19" s="11">
+        <v>2</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:P18">
+  <conditionalFormatting sqref="C5:P19">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"non"</formula>
     </cfRule>

</xml_diff>